<commit_message>
Campagne LinkedIn : formulaire /avis/, visuels, dates et lien réel dans le kit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0115fun8orvgDhHD6MW8HSV5
</commit_message>
<xml_diff>
--- a/ready-to-reply/validation-linkedin/ready-to-reply-suivi-validation-linkedin.xlsx
+++ b/ready-to-reply/validation-linkedin/ready-to-reply-suivi-validation-linkedin.xlsx
@@ -853,7 +853,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
+      <c r="A2" s="5" t="n">
+        <v>46301</v>
+      </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
           <t>P1 · Le problème</t>
@@ -878,7 +880,9 @@
       <c r="O2" s="7" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
+      <c r="A3" s="5" t="n">
+        <v>46308</v>
+      </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
           <t>P2 · Les conséquences</t>
@@ -903,7 +907,9 @@
       <c r="O3" s="7" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
+      <c r="A4" s="5" t="n">
+        <v>46315</v>
+      </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>P3 · L'idée de Ready To Reply</t>
@@ -928,7 +934,9 @@
       <c r="O4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
+      <c r="A5" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
           <t>P4 · Invitation à échanger</t>

</xml_diff>